<commit_message>
working on prelim figs
</commit_message>
<xml_diff>
--- a/01_Raw_data/stream dims.xlsx
+++ b/01_Raw_data/stream dims.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Howley_Bradford_Streams\Howley_Bradford_Streams\01_Raw_data\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9DB9255C-703A-4E6E-8274-81FDECEA71E2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CA5E8EC0-A70D-45A7-AB42-DCA0097FBBF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="10260" xr2:uid="{3BE57CE1-FABC-4E3B-A6CB-89ECB7AEEF69}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{3BE57CE1-FABC-4E3B-A6CB-89ECB7AEEF69}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Long site" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="191029"/>
   <extLst>
@@ -36,7 +37,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="6" uniqueCount="6">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="42" uniqueCount="16">
   <si>
     <t>ID</t>
   </si>
@@ -54,6 +55,36 @@
   </si>
   <si>
     <t>UCA</t>
+  </si>
+  <si>
+    <t>UCA_km</t>
+  </si>
+  <si>
+    <t>9</t>
+  </si>
+  <si>
+    <t>0</t>
+  </si>
+  <si>
+    <t>4</t>
+  </si>
+  <si>
+    <t>3</t>
+  </si>
+  <si>
+    <t>2</t>
+  </si>
+  <si>
+    <t>1</t>
+  </si>
+  <si>
+    <t>5</t>
+  </si>
+  <si>
+    <t>6</t>
+  </si>
+  <si>
+    <t>Long</t>
   </si>
 </sst>
 </file>
@@ -425,10 +456,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1C404516-DA56-45A0-8A9A-A195294C582E}">
-  <dimension ref="A1:D10"/>
+  <dimension ref="A1:E10"/>
   <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
   <sheetData>
-    <row r="1" spans="1:4" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -441,8 +472,11 @@
       <c r="D1" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="2" spans="1:4" x14ac:dyDescent="0.75">
+      <c r="E1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A2">
         <v>5</v>
       </c>
@@ -457,7 +491,7 @@
         <v>2.0000000000000001E-4</v>
       </c>
     </row>
-    <row r="3" spans="1:4" x14ac:dyDescent="0.75">
+    <row r="3" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A3" t="s">
         <v>1</v>
       </c>
@@ -465,7 +499,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="4" spans="1:4" x14ac:dyDescent="0.75">
+    <row r="4" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A4">
         <v>15</v>
       </c>
@@ -477,7 +511,7 @@
         <v>2.4384000000000001</v>
       </c>
     </row>
-    <row r="5" spans="1:4" x14ac:dyDescent="0.75">
+    <row r="5" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A5">
         <v>3</v>
       </c>
@@ -485,7 +519,7 @@
         <v>2.72</v>
       </c>
     </row>
-    <row r="6" spans="1:4" x14ac:dyDescent="0.75">
+    <row r="6" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A6">
         <v>7</v>
       </c>
@@ -497,7 +531,7 @@
         <v>6.0960000000000001</v>
       </c>
     </row>
-    <row r="7" spans="1:4" x14ac:dyDescent="0.75">
+    <row r="7" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A7">
         <v>6</v>
       </c>
@@ -508,7 +542,7 @@
         <v>1.4E-3</v>
       </c>
     </row>
-    <row r="8" spans="1:4" x14ac:dyDescent="0.75">
+    <row r="8" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A8" t="s">
         <v>2</v>
       </c>
@@ -516,7 +550,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="9" spans="1:4" x14ac:dyDescent="0.75">
+    <row r="9" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A9">
         <v>9</v>
       </c>
@@ -527,7 +561,7 @@
         <v>2.9999999999999997E-4</v>
       </c>
     </row>
-    <row r="10" spans="1:4" x14ac:dyDescent="0.75">
+    <row r="10" spans="1:5" x14ac:dyDescent="0.75">
       <c r="A10">
         <v>13</v>
       </c>
@@ -537,6 +571,203 @@
       <c r="C10">
         <f t="shared" si="0"/>
         <v>4.2671999999999999</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{BAFDE701-703F-4A4B-B715-D05CA66634AD}">
+  <dimension ref="A1:C17"/>
+  <sheetFormatPr defaultRowHeight="14.75" x14ac:dyDescent="0.75"/>
+  <sheetData>
+    <row r="1" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C1" t="s">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A2" t="s">
+        <v>7</v>
+      </c>
+      <c r="B2" t="s">
+        <v>8</v>
+      </c>
+      <c r="C2">
+        <v>19864100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A3" t="s">
+        <v>7</v>
+      </c>
+      <c r="B3" t="s">
+        <v>9</v>
+      </c>
+      <c r="C3">
+        <v>19268200</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A4" t="s">
+        <v>7</v>
+      </c>
+      <c r="B4" t="s">
+        <v>10</v>
+      </c>
+      <c r="C4">
+        <v>5821280</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A5" t="s">
+        <v>7</v>
+      </c>
+      <c r="B5" t="s">
+        <v>11</v>
+      </c>
+      <c r="C5">
+        <v>1960760</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A6" t="s">
+        <v>7</v>
+      </c>
+      <c r="B6" t="s">
+        <v>12</v>
+      </c>
+      <c r="C6">
+        <v>262193</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A7" t="s">
+        <v>13</v>
+      </c>
+      <c r="B7" t="s">
+        <v>8</v>
+      </c>
+      <c r="C7">
+        <v>17795000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A8" t="s">
+        <v>13</v>
+      </c>
+      <c r="B8" t="s">
+        <v>9</v>
+      </c>
+      <c r="C8">
+        <v>14519100</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A9" t="s">
+        <v>13</v>
+      </c>
+      <c r="B9" t="s">
+        <v>10</v>
+      </c>
+      <c r="C9">
+        <v>10249400</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A10" t="s">
+        <v>13</v>
+      </c>
+      <c r="B10" t="s">
+        <v>11</v>
+      </c>
+      <c r="C10">
+        <v>1812340</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A11" t="s">
+        <v>13</v>
+      </c>
+      <c r="B11" t="s">
+        <v>12</v>
+      </c>
+      <c r="C11">
+        <v>138375</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A12" t="s">
+        <v>10</v>
+      </c>
+      <c r="B12" t="s">
+        <v>12</v>
+      </c>
+      <c r="C12">
+        <v>9204</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A13" t="s">
+        <v>10</v>
+      </c>
+      <c r="B13" t="s">
+        <v>11</v>
+      </c>
+      <c r="C13">
+        <v>1355500</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A14" t="s">
+        <v>10</v>
+      </c>
+      <c r="B14" t="s">
+        <v>9</v>
+      </c>
+      <c r="C14">
+        <v>1139580</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A15" t="s">
+        <v>14</v>
+      </c>
+      <c r="B15" t="s">
+        <v>12</v>
+      </c>
+      <c r="C15">
+        <v>3131520</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A16" t="s">
+        <v>14</v>
+      </c>
+      <c r="B16" t="s">
+        <v>11</v>
+      </c>
+      <c r="C16">
+        <v>26276900</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" x14ac:dyDescent="0.75">
+      <c r="A17" t="s">
+        <v>14</v>
+      </c>
+      <c r="B17" t="s">
+        <v>10</v>
+      </c>
+      <c r="C17">
+        <v>26315900</v>
       </c>
     </row>
   </sheetData>

</xml_diff>